<commit_message>
Con Law chart: add National Pork Producers handout vote map and notes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBALxAraNGVe1dMDEfigDw
</commit_message>
<xml_diff>
--- a/Con_Law_Case_Chart.xlsx
+++ b/Con_Law_Case_Chart.xlsx
@@ -8691,7 +8691,7 @@
       </c>
       <c r="H149" s="3" t="inlineStr">
         <is>
-          <t>Affirmed: the complaint fails to state a dormant Commerce Clause claim. The Court unanimously rejects an "almost per se" rule against state laws with extraterritorial effects; a fractured majority rejects the Pike claim.</t>
+          <t>Affirmed (Ninth Circuit): the complaint fails to state a dormant Commerce Clause claim. All nine Justices reject an "almost per se" rule against state laws with extraterritorial effects (Part III: 5-Justice majority, with Roberts, Alito, Kavanaugh and Jackson agreeing). The Pike claim fails on a fractured vote: IV-C's no-substantial-burden reasoning has only 4 votes, and IV-B's incommensurability reasoning only 3.</t>
         </is>
       </c>
       <c r="I149" s="3" t="inlineStr">
@@ -8701,19 +8701,25 @@
       </c>
       <c r="J149" s="3" t="inlineStr">
         <is>
-          <t>• Gorsuch for the Court (Parts I-III, IV-A, V): no extraterritoriality rule; Pike's heartland = discrimination
-• Part IV-B (Gorsuch, Thomas, Barrett): courts can't weigh economic costs against moral/health benefits; "incommensurable" ("whether a particular line is longer than a particular rock is heavy"); take it to Congress
-• Part IV-C (Gorsuch, Thomas, Sotomayor, Kagan): no substantial burden pled; Exxon analogy (market share shifts among out-of-state firms; "That goes for pigs no less than gas stations")
-• Sotomayor (with Kagan): Pike survives; courts CAN balance; claim fails only for no substantial burden
-• Barrett: burdens are substantial, but benefits and burdens are incommensurable
-• Roberts (with Alito, Kavanaugh, Jackson), partial dissent: substantial burden pled (market-wide harms, compliance forced even on producers not selling in CA, Edgar's "nationwide reach"); would remand for Pike balancing
-• Kavanaugh: six Justices keep Pike balancing; Prop 12 may also raise Import-Export, Privileges and Immunities and Full Faith and Credit issues; "California knows best"
-• Count: 6 Justices say courts can balance under Pike; the judgment rests on IV-B + IV-C together</t>
+          <t>• VOTE MAP (handout), Gorsuch's lead opinion: I Facts (5: NG/CT/SS/EK/ACB)
+• II No discrimination (5)
+• III No per se extraterritoriality rule (5, + JR/SA/BK/KBJ in agreement = 9)
+• IV-A No clear line between discrimination and Pike cases (5; Roberts seemed to agree that many leading dormant CC cases are really about protectionism)
+• IV-B Incommensurability: courts can't weigh economic costs against moral/health benefits ("whether a particular line is longer than a particular rock is heavy") (3: NG/CT/ACB; 6 disagree: SS/EK + JR/SA/BK/KBJ)
+• IV-C Pike pleading requirement not met: no substantial burden pled; Exxon analogy ("That goes for pigs no less than gas stations") (4: NG/CT/SS/EK; 5 disagree: ACB + JR/SA/BK/KBJ)
+• IV-D Federalism + incommensurability (3: NG/CT/ACB; 6 implicitly disagree)
+• V Judgment affirmed (5)
+• IS THE OPINION FRACTURED? Gorsuch/Thomas/Barrett say no (the dissents "seek to characterize today's decision as 'fractured'"); everyone else says yes
+• IS PIKE OVERRULED? No. Kavanaugh: IV-B and IV-D "would essentially overrule the Pike balancing test," but "six Justices of this Court affirmatively retain" it (SS, EK + JR, SA, BK, KBJ)
+• WHAT'S BINDING? Majority parts: I, II, III, IV-A, V. Gorsuch (IV-D) claims the judgment "depends equally" on IV-B and IV-C; Kavanaugh: IV-B and IV-D "are not controlling precedent," but IV-C (4-Justice plurality applying Pike) is controlling for the judgment on the Pike claim
+• FIVE Justices think a substantial burden WAS pled: Barrett ("The complaint plausibly alleges that Proposition 12's costs are pervasive, burdensome, and will be felt primarily (but not exclusively) outside California"; so she doesn't join IV-C, but votes to affirm on incommensurability) + Roberts/Alito/Kavanaugh/Jackson (would remand for Pike balancing)
+• FEDERALISM CUTS BOTH WAYS: Gorsuch/Thomas/Barrett (IV-D): the dissent's test means "one complaint from an unhappy out-of-state producer and—presto—the Constitution would protect the sale of horsemeat" (also fireworks, plastic bags); Kavanaugh: California "undermines federalism" by forcing other States' farmers to follow its laws
+• Kavanaugh also flags Import-Export, Privileges and Immunities and Full Faith and Credit issues</t>
         </is>
       </c>
       <c r="K149" s="3" t="inlineStr">
         <is>
-          <t>Modern statement that the dormant CC is about discrimination. For a facially neutral law, walk the Truesdell questions (face, effect, purpose), then Pike: substantial burden first, then 'clearly excessive' balancing. Shows the Court's caution: leave nationwide policy to Congress under the 'wakeful' Commerce Clause.</t>
+          <t>Modern statement that the dormant CC is about discrimination. For a facially neutral law, walk the Truesdell questions (face, effect, purpose), then Pike: substantial burden first, then 'clearly excessive' balancing. Count votes carefully: Pike balancing survives (6 Justices), the extraterritoriality argument is dead (9), and the binding Pike holding is at most IV-C's narrow pleading point. Argue federalism from both sides (horsemeat vs. California dictating farm practices). The Court leaves nationwide policy to Congress under the 'wakeful' Commerce Clause.</t>
         </is>
       </c>
     </row>
@@ -14882,7 +14888,7 @@
       </c>
       <c r="F116" s="3" t="inlineStr">
         <is>
-          <t>Affirmed: the complaint fails to state a dormant Commerce Clause claim. The Court unanimously rejects an "almost per se" rule against state laws with extraterritorial effects; a fractured majority rejects the Pike claim.</t>
+          <t>Affirmed (Ninth Circuit): the complaint fails to state a dormant Commerce Clause claim. All nine Justices reject an "almost per se" rule against state laws with extraterritorial effects (Part III: 5-Justice majority, with Roberts, Alito, Kavanaugh and Jackson agreeing). The Pike claim fails on a fractured vote: IV-C's no-substantial-burden reasoning has only 4 votes, and IV-B's incommensurability reasoning only 3.</t>
         </is>
       </c>
       <c r="G116" s="3" t="inlineStr">
@@ -14892,19 +14898,25 @@
       </c>
       <c r="H116" s="3" t="inlineStr">
         <is>
-          <t>• Gorsuch for the Court (Parts I-III, IV-A, V): no extraterritoriality rule; Pike's heartland = discrimination
-• Part IV-B (Gorsuch, Thomas, Barrett): courts can't weigh economic costs against moral/health benefits; "incommensurable" ("whether a particular line is longer than a particular rock is heavy"); take it to Congress
-• Part IV-C (Gorsuch, Thomas, Sotomayor, Kagan): no substantial burden pled; Exxon analogy (market share shifts among out-of-state firms; "That goes for pigs no less than gas stations")
-• Sotomayor (with Kagan): Pike survives; courts CAN balance; claim fails only for no substantial burden
-• Barrett: burdens are substantial, but benefits and burdens are incommensurable
-• Roberts (with Alito, Kavanaugh, Jackson), partial dissent: substantial burden pled (market-wide harms, compliance forced even on producers not selling in CA, Edgar's "nationwide reach"); would remand for Pike balancing
-• Kavanaugh: six Justices keep Pike balancing; Prop 12 may also raise Import-Export, Privileges and Immunities and Full Faith and Credit issues; "California knows best"
-• Count: 6 Justices say courts can balance under Pike; the judgment rests on IV-B + IV-C together</t>
+          <t>• VOTE MAP (handout), Gorsuch's lead opinion: I Facts (5: NG/CT/SS/EK/ACB)
+• II No discrimination (5)
+• III No per se extraterritoriality rule (5, + JR/SA/BK/KBJ in agreement = 9)
+• IV-A No clear line between discrimination and Pike cases (5; Roberts seemed to agree that many leading dormant CC cases are really about protectionism)
+• IV-B Incommensurability: courts can't weigh economic costs against moral/health benefits ("whether a particular line is longer than a particular rock is heavy") (3: NG/CT/ACB; 6 disagree: SS/EK + JR/SA/BK/KBJ)
+• IV-C Pike pleading requirement not met: no substantial burden pled; Exxon analogy ("That goes for pigs no less than gas stations") (4: NG/CT/SS/EK; 5 disagree: ACB + JR/SA/BK/KBJ)
+• IV-D Federalism + incommensurability (3: NG/CT/ACB; 6 implicitly disagree)
+• V Judgment affirmed (5)
+• IS THE OPINION FRACTURED? Gorsuch/Thomas/Barrett say no (the dissents "seek to characterize today's decision as 'fractured'"); everyone else says yes
+• IS PIKE OVERRULED? No. Kavanaugh: IV-B and IV-D "would essentially overrule the Pike balancing test," but "six Justices of this Court affirmatively retain" it (SS, EK + JR, SA, BK, KBJ)
+• WHAT'S BINDING? Majority parts: I, II, III, IV-A, V. Gorsuch (IV-D) claims the judgment "depends equally" on IV-B and IV-C; Kavanaugh: IV-B and IV-D "are not controlling precedent," but IV-C (4-Justice plurality applying Pike) is controlling for the judgment on the Pike claim
+• FIVE Justices think a substantial burden WAS pled: Barrett ("The complaint plausibly alleges that Proposition 12's costs are pervasive, burdensome, and will be felt primarily (but not exclusively) outside California"; so she doesn't join IV-C, but votes to affirm on incommensurability) + Roberts/Alito/Kavanaugh/Jackson (would remand for Pike balancing)
+• FEDERALISM CUTS BOTH WAYS: Gorsuch/Thomas/Barrett (IV-D): the dissent's test means "one complaint from an unhappy out-of-state producer and—presto—the Constitution would protect the sale of horsemeat" (also fireworks, plastic bags); Kavanaugh: California "undermines federalism" by forcing other States' farmers to follow its laws
+• Kavanaugh also flags Import-Export, Privileges and Immunities and Full Faith and Credit issues</t>
         </is>
       </c>
       <c r="I116" s="3" t="inlineStr">
         <is>
-          <t>Modern statement that the dormant CC is about discrimination. For a facially neutral law, walk the Truesdell questions (face, effect, purpose), then Pike: substantial burden first, then 'clearly excessive' balancing. Shows the Court's caution: leave nationwide policy to Congress under the 'wakeful' Commerce Clause.</t>
+          <t>Modern statement that the dormant CC is about discrimination. For a facially neutral law, walk the Truesdell questions (face, effect, purpose), then Pike: substantial burden first, then 'clearly excessive' balancing. Count votes carefully: Pike balancing survives (6 Justices), the extraterritoriality argument is dead (9), and the binding Pike holding is at most IV-C's narrow pleading point. Argue federalism from both sides (horsemeat vs. California dictating farm practices). The Court leaves nationwide policy to Congress under the 'wakeful' Commerce Clause.</t>
         </is>
       </c>
     </row>

</xml_diff>